<commit_message>
docs(acta): ronda 28/09-02/10 -- filas 58-62 de KomfIA, encabezado al 02/10
Feedback de flota, rendimiento, comandos, pedidos de gerencia (tabla unica,
panel, historiales) y los hallazgos de datos para el area. Editada por XML
directo; logo y 215 checkboxes intactos; sincronizada con INVERTEX v3.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/gerencia/ACTA DE REUNION_PROYECTOS DE DESARROLLO CONFIABILIDAD.xlsx
+++ b/docs/gerencia/ACTA DE REUNION_PROYECTOS DE DESARROLLO CONFIABILIDAD.xlsx
@@ -930,8 +930,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla2" displayName="Tabla2" ref="B19:K57" totalsRowShown="0" headerRowDxfId="14" dataDxfId="12" headerRowBorderDxfId="13" tableBorderDxfId="11" totalsRowBorderDxfId="10">
-  <autoFilter ref="B19:K57" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla2" displayName="Tabla2" ref="B19:K62" totalsRowShown="0" headerRowDxfId="14" dataDxfId="12" headerRowBorderDxfId="13" tableBorderDxfId="11" totalsRowBorderDxfId="10">
+  <autoFilter ref="B19:K62" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Proyecto" dataDxfId="9"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Asunto" dataDxfId="8"/>
@@ -1265,7 +1265,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:K57"/>
+  <dimension ref="B2:K62"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.77734375" customWidth="1"/>
@@ -1303,7 +1303,7 @@
         <v>17</v>
       </c>
       <c r="K4" s="8">
-        <v>46283</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.3">
@@ -2983,7 +2983,7 @@
         </is>
       </c>
     </row>
-    <row r="57" spans="2:11" ht="245" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:11" ht="260" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B57" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">KomfIA</t>
@@ -3021,7 +3021,236 @@
         <is>
           <t xml:space="preserve">25/09/26 - Las 14 observaciones y los arreglos de esta ronda fueron sobre los módulos de un equipo: último análisis, condición de motores de tracción, diagnóstico, tendencia, gráfica, historial y acumulados.
 25/09/26 - Los módulos de flota (barrido, triage, conteo, rankings, tendencia incipiente) NO fueron revisados con el área en esta ronda. Se espera feedback sobre ellos en una próxima sesión.
-25/09/26 - Notificado a Carlos: las pruebas nuevas son sobre los módulos POR EQUIPO. El feedback de los módulos POR FLOTA queda para una sesión posterior.</t>
+25/09/26 - Notificado a Carlos: las pruebas nuevas son sobre los módulos POR EQUIPO. El feedback de los módulos POR FLOTA queda para una sesión posterior.
+28/09/26 - Llegó el feedback de los módulos de flota: ver filas 58 a 62.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" spans="2:11" ht="295" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B58" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KomfIA</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ronda de feedback 28/09 — módulos de flota y límites completos</t>
+        </is>
+      </c>
+      <c r="D58" s="8">
+        <v>46293</v>
+      </c>
+      <c r="E58" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Atender el feedback de la revisión del 28/09, centrada en los módulos POR FLOTA, y que todos los módulos usen los límites completos del área.</t>
+        </is>
+      </c>
+      <c r="F58" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="G58" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="H58" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="I58" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="J58" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="K58" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">28/09/26 - Feedback recibido (Carlos y gerencia) sobre los módulos de flota: barrido, triage, conteo, rankings, tendencia incipiente, gráfica e historial.
+29/09/26 - Límites: la base tiene 38 parámetros con límite y el sistema leía 16. Ahora lee los 38 (fósforo, boro, viscosidad, ISO, TAN, hollín, agua…): desaparecen los «—» que señalaba Carlos.
+29/09/26 - Triage con 5 columnas por familia (Desgaste · Aditivos · Contaminación · Salud · Cód. Limpieza), cada parámetro con su valor.
+29/09/26 - Un valor 0 del laboratorio ya no se toma como medición: fabricaba críticos en aditivos y daba por limpios componentes que no se midieron.
+30/09/26 - El filtro por modelo ahora llega a la base: «/barrido antapaccay 980» muestra solo los 980E. Antes lo filtraba la IA, a veces sí y a veces no.
+30/09/26 - Barrido de Antamina: marcaba Ca/Zn/Mg en rojo en el 100 % de ruedas e hidráulicos por evaluar el aditivo al revés. Corregido; ahora coincide con el triage.
+30/09/26 - La IA de respaldo ya no arma tablas propias (se confundían con las reales): responde en viñetas, marcadas con 🔎.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" spans="2:11" ht="190" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B59" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KomfIA</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rendimiento — fin de los tiempos de espera en producción</t>
+        </is>
+      </c>
+      <c r="D59" s="8">
+        <v>46295</v>
+      </c>
+      <c r="E59" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Que ningún módulo por equipo exceda el tiempo de Teams, y dejar documentado el método para repetirlo.</t>
+        </is>
+      </c>
+      <c r="F59" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="G59" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="H59" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="I59" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="J59" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="K59" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30/09/26 - Detectado en la prueba en Teams: el diagnóstico completo y la condición de motores de tracción no respondían (tiempo agotado, ~170 s y ~146 s).
+30/09/26 - Causa: las consultas calculaban la flota entera y recién al final filtraban el equipo. Reestructuradas para filtrar primero.
+30/09/26 - Resultado: condición MT 146 s -&gt; 1,4 s · diagnóstico completo 170 s -&gt; 6,6 s · otras 7 consultas mejoradas. Sin índices nuevos ni cambios en la base.
+30/09/26 - El método quedó documentado como procedimiento interno de diagnóstico.
+02/10/26 - PENDIENTE (no urgente): la tendencia (~33 s) y los tres historiales (~34 s) responden, pero se pueden acelerar con el mismo método.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" spans="2:11" ht="160" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B60" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KomfIA</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Comandos — el sistema pregunta lo que falta</t>
+        </is>
+      </c>
+      <c r="D60" s="8">
+        <v>46295</v>
+      </c>
+      <c r="E60" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Que cada comando funcione aunque falten datos (los pide), acepte las distintas formas del código del camión y no se desvíe a otro módulo.</t>
+        </is>
+      </c>
+      <c r="F60" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="G60" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="H60" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="I60" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="J60" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="K60" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30/09/26 - /barrido y /ranking aceptan el modelo (980E, D475A…).
+01/10/26 - 11 módulos preguntan lo que falta (equipo, componente, metal) en lugar de responder «No encontré datos». Ej.: «/ranking» pide el componente y el metal.
+01/10/26 - Código de Cummins: «T3160» encuentra el CA3160, igual que «3160» y «CA3160».
+01/10/26 - /grafica absorbe /tendenciametal: un comando menos. «/triage antapaccay» funciona escribiendo primero la mina.
+02/10/26 - Los comandos ya no se desvían a otro módulo por coincidir en el nombre (ej. /barrido caía en el detalle).</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" spans="2:11" ht="190" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B61" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KomfIA</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pedidos de gerencia — tabla única, panel de flota e historial completo</t>
+        </is>
+      </c>
+      <c r="D61" s="8">
+        <v>46293</v>
+      </c>
+      <c r="E61" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aplicar los pedidos de forma del 28/09 y 01/10: una sola tabla en tendencia y gráfica, un panel de la mina en lugar del barrido resumen, e historiales con todos los parámetros.</t>
+        </is>
+      </c>
+      <c r="F61" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="G61" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="H61" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="I61" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="J61" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="K61" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">01/10/26 - Tendencia y gráfica en UNA sola tabla (antes eran dos con las mismas fechas). En la gráfica, la fila del metal va primero.
+01/10/26 - Diagnóstico: el SMR (horómetro) arriba, y las filas Fecha última · Horas de componente · Tipo de muestra de cada componente.
+02/10/26 - /panel (también /barrido y /conteo): cómo está la mina — equipos, observados, por componente con «lo que más se repite», por modelo y por dónde empezar. Cuadra exacto con el conteo anterior.
+02/10/26 - Historial de componente y de equipo: en lugar de «Met. Obs.», las 5 familias del formato con su valor («Fe (232.6)»). Se mantiene vertical: Teams no hace scroll horizontal.
+02/10/26 - Historial de flota: cada parámetro con su valor y el componente en mayúsculas; toda fila observada nombra lo que la marcó.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" spans="2:11" ht="220" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B62" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KomfIA</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hallazgos de datos para el área (próximo feedback)</t>
+        </is>
+      </c>
+      <c r="D62" s="8">
+        <v>46297</v>
+      </c>
+      <c r="E62" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Llevar al área lo que el sistema ya muestra correctamente pero depende de la carga de datos o de los límites cargados.</t>
+        </is>
+      </c>
+      <c r="F62" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="G62" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="H62" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="I62" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="J62" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="K62" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">02/10/26 - Para revisar con Carlos (no es del sistema: es carga o límites):
+1. Ruedas de Antapaccay: el límite se escribió para otro aceite (Mobiltrans) y las ruedas corren Spirax.
+2. 885 componentes sin ningún límite cargado: salen sin evaluar.
+3. 347 componentes con ISO en 0 (sin medir).
+4. 1 579 muestras de Cerro Verde sin componente.
+5. Antamina: Ca/Zn/Mg sin límite de precaución (solo existe el crítico).
+6. Error de tipeo «MOTORO DE TRACCION RH»: sigue entrando.
+7. Componente cargado como «nan».
+8. HT301 RD LH (10/09): probable muestra mal rotulada.
+9. Viscosidad (V100) en rojo en casi todas las ruedas de Antamina.
+10. Decisión: ¿el código ISO debe contar como observado? Hoy el triage y los historiales lo cuentan; el panel y el barrido no.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: cierre de la ronda 03/10 -- acta filas 63-64, PENDIENTES limpio (8 abiertos), avance semanal 28/09, conteos y CONFIG al dia
- acta: presentacion de la alfa (02/10) y rendimiento; K4 = 03/10; copia sincronizada en INVERTEX
- PENDIENTES: ronda R1-R16 archivada en pendientes-legado/PENDIENTES_2026-10-03.md
- CONFIG_TEMAS (13/14 via MD_historial), CONFIG_FLUJOS, CONFIG_TIMEOUT, PRUEBAS_ALFA (N11), BITACORA, README, ESQUEMA_BD (12 vistas fuera del Excel)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/gerencia/ACTA DE REUNION_PROYECTOS DE DESARROLLO CONFIABILIDAD.xlsx
+++ b/docs/gerencia/ACTA DE REUNION_PROYECTOS DE DESARROLLO CONFIABILIDAD.xlsx
@@ -930,8 +930,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla2" displayName="Tabla2" ref="B19:K62" totalsRowShown="0" headerRowDxfId="14" dataDxfId="12" headerRowBorderDxfId="13" tableBorderDxfId="11" totalsRowBorderDxfId="10">
-  <autoFilter ref="B19:K62" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla2" displayName="Tabla2" ref="B19:K64" totalsRowShown="0" headerRowDxfId="14" dataDxfId="12" headerRowBorderDxfId="13" tableBorderDxfId="11" totalsRowBorderDxfId="10">
+  <autoFilter ref="B19:K64" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Proyecto" dataDxfId="9"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Asunto" dataDxfId="8"/>
@@ -1265,7 +1265,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:K62"/>
+  <dimension ref="B2:K64"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.77734375" customWidth="1"/>
@@ -1303,7 +1303,7 @@
         <v>17</v>
       </c>
       <c r="K4" s="8">
-        <v>46297</v>
+        <v>46298</v>
       </c>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.3">
@@ -3072,7 +3072,7 @@
         </is>
       </c>
     </row>
-    <row r="59" spans="2:11" ht="190" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:11" ht="210" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B59" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">KomfIA</t>
@@ -3112,7 +3112,8 @@
 30/09/26 - Causa: las consultas calculaban la flota entera y recién al final filtraban el equipo. Reestructuradas para filtrar primero.
 30/09/26 - Resultado: condición MT 146 s -&gt; 1,4 s · diagnóstico completo 170 s -&gt; 6,6 s · otras 7 consultas mejoradas. Sin índices nuevos ni cambios en la base.
 30/09/26 - El método quedó documentado como procedimiento interno de diagnóstico.
-02/10/26 - PENDIENTE (no urgente): la tendencia (~33 s) y los tres historiales (~34 s) responden, pero se pueden acelerar con el mismo método.</t>
+02/10/26 - PENDIENTE (no urgente): la tendencia (~33 s) y los tres historiales (~34 s) responden, pero se pueden acelerar con el mismo método.
+03/10/26 - Resuelto: la tendencia bajó a 19 s y los historiales a entre 0,5 y 10 s (ver fila 64).</t>
         </is>
       </c>
     </row>
@@ -3251,6 +3252,95 @@
 8. HT301 RD LH (10/09): probable muestra mal rotulada.
 9. Viscosidad (V100) en rojo en casi todas las ruedas de Antamina.
 10. Decisión: ¿el código ISO debe contar como observado? Hoy el triage y los historiales lo cuentan; el panel y el barrido no.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" spans="2:11" ht="280" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B63" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KomfIA</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Presentación de la alfa a gerencia (02/10) — límites y alerta temprana</t>
+        </is>
+      </c>
+      <c r="D63" s="8">
+        <v>46297</v>
+      </c>
+      <c r="E63" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Corregir lo que se vio en la primera presentación de la alfa: límites que no aparecían y una alerta temprana que no detectó un caso real.</t>
+        </is>
+      </c>
+      <c r="F63" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="G63" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="H63" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="I63" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="J63" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="K63" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">02/10/26 - Presentación de la alfa a gerencia. Equipo testigo: CA3195, motor de tracción LH, con PQ 233 en su última muestra.
+03/10/26 - Límites: el último análisis y la tendencia no mostraban los límites de aditivos (P, B), viscosidad ni código de limpieza, aunque Antapaccay sí los tiene cargados. Corregido: todos los parámetros con su límite.
+03/10/26 - El código de limpieza (ISO) se muestra siempre en enteros, como corresponde a un código.
+03/10/26 - La fila «Estado» de la tendencia ahora coincide con la del historial (antes una misma muestra salía verde en una y roja en la otra).
+03/10/26 - Alerta temprana (/incipiente): no listaba al CA3195 porque descartaba lo que ya había pasado el límite. Nueva categoría «cruzó»: lo que pasa el límite viniendo de valores normales. El CA3195 sale primero. Acepta el modelo (/incipiente antapaccay 980) y muestra los límites de cada modelo.
+03/10/26 - Otros: /historial con el componente escrito junto («MTLH») ya funciona; /triage con un equipo lleva al diagnóstico de ese equipo; /historialmetal de P o B ya no mezcla otros metales.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" spans="2:11" ht="220" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B64" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KomfIA</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rendimiento — por qué se demoró la presentación y la corrección</t>
+        </is>
+      </c>
+      <c r="D64" s="8">
+        <v>46298</v>
+      </c>
+      <c r="E64" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Explicar los tiempos de espera del 02/10 y evitar que se repitan.</t>
+        </is>
+      </c>
+      <c r="F64" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="G64" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="H64" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="I64" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="J64" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="K64" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">03/10/26 - Causa medida: la base de datos tiene un tope de procesamiento (el plan contratado) y las consultas que corren a la vez se lo reparten. El 02/10 se sumaron reintentos automáticos (una consulta repetida 4 veces) y consultas abandonadas que seguían corriendo.
+03/10/26 - Corregido: reintentos desactivados en los flujos. Alerta temprana 10 s -&gt; 2 s; tendencia 32 s -&gt; 19 s; historiales de 34-80 s a entre 0,5 y 10 s, con exactamente el mismo resultado.
+03/10/26 - Para revisar con TI: un permiso de solo lectura de métricas (VIEW DATABASE PERFORMANCE STATE) para ver qué pasó en la base en un momento dado, y evaluar el plan de la base.
+PENDIENTE a largo plazo: comando /limites (la tabla de límites que usa el semáforo). Listo en la base, sin publicar.
+EN ESTUDIO: una ponderación por parámetro, relacionada al ranking de acumulados; el código de limpieza podría entrar ahí.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(acta): filas 65-66 -- flujo de uso de Carlos cableado de punta a punta y pendientes al 04/10; encabezado al 04/10
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/gerencia/ACTA DE REUNION_PROYECTOS DE DESARROLLO CONFIABILIDAD.xlsx
+++ b/docs/gerencia/ACTA DE REUNION_PROYECTOS DE DESARROLLO CONFIABILIDAD.xlsx
@@ -930,8 +930,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla2" displayName="Tabla2" ref="B19:K64" totalsRowShown="0" headerRowDxfId="14" dataDxfId="12" headerRowBorderDxfId="13" tableBorderDxfId="11" totalsRowBorderDxfId="10">
-  <autoFilter ref="B19:K64" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla2" displayName="Tabla2" ref="B19:K66" totalsRowShown="0" headerRowDxfId="14" dataDxfId="12" headerRowBorderDxfId="13" tableBorderDxfId="11" totalsRowBorderDxfId="10">
+  <autoFilter ref="B19:K66" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Proyecto" dataDxfId="9"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Asunto" dataDxfId="8"/>
@@ -1265,7 +1265,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:K64"/>
+  <dimension ref="B2:K66"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.77734375" customWidth="1"/>
@@ -1303,7 +1303,7 @@
         <v>17</v>
       </c>
       <c r="K4" s="8">
-        <v>46298</v>
+        <v>46299</v>
       </c>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.3">
@@ -3344,6 +3344,96 @@
         </is>
       </c>
     </row>
+    <row r="65" spans="2:11" ht="265" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B65" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KomfIA</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Flujo de uso de Carlos (reunión 02/10) — cableado de punta a punta</t>
+        </is>
+      </c>
+      <c r="D65" s="8">
+        <v>46297</v>
+      </c>
+      <c r="E65" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Que el recorrido de análisis que definió Carlos funcione completo, de la mina al metal, sin perder parámetros en ningún paso.</t>
+        </is>
+      </c>
+      <c r="F65" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="G65" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="H65" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="I65" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="J65" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="K65" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">02/10/26 - En la reunión, Carlos definió su flujo de uso. MACRO: barrido detalle → alerta temprana → ranking o triage → historial de flota. MICRO: diagnóstico del equipo → condición MT (LH vs RH) → último análisis → tendencia → gráfica → historiales.
+04/10/26 - Todos los módulos muestran el formato completo: el código de limpieza (ISO), P, B y Mo ya aparecen en el barrido detalle, la condición MT, el último por metal y el ranking (lo que faltaba en el CA3195).
+04/10/26 - Un comando de flota que recibe un equipo (ej. «/barridodet 3195») lleva directo al análisis de ese equipo.
+04/10/26 - Barrido detalle ordenado: MT LH, MT RH, sistema hidráulico, motor, rueda LH, rueda RH; su tabla de límites incluye ahora todos los parámetros marcados.
+04/10/26 - Rendimiento: barrido detalle 18 s → 2 s; historiales ~10 s → menos de 1 s; condición MT, historial de flota y alerta temprana en 2-3 s.
+04/10/26 - Prueba completa en Teams con el CA3195, de la mina al metal: funciona de punta a punta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" spans="2:11" ht="220" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B66" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KomfIA</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pendientes al 04/10</t>
+        </is>
+      </c>
+      <c r="D66" s="8">
+        <v>46299</v>
+      </c>
+      <c r="E66" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lo que queda abierto tras la ronda de la presentación del 02/10.</t>
+        </is>
+      </c>
+      <c r="F66" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="G66" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="H66" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="I66" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="J66" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="K66" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Con Carlos (próximo feedback): los hallazgos de carga y límites de la fila 64 (ruedas con límite de otro aceite, componentes sin límites, ISO en 0, etc.) y si el «Acum» del PQ tiene sentido.
+En estudio: ponderación por parámetro (ligada al ranking de acumulados); decide si el código de limpieza cuenta para el estado en el panel y el barrido.
+Rendimiento: el diagnóstico completo aún lee la base 7 veces (7-11 s); es el último ajuste del flujo de uso.
+Copilot: la conexión SQL de algunos flujos queda «obsoleta» durante las pruebas y Teams pide reconectar.
+TI / DBA: permiso de solo lectura de métricas (VIEW DATABASE PERFORMANCE STATE) y evaluar el plan de la base.
+A largo plazo: comando /limites, «siguiente paso sugerido» al pie de los módulos de flota y pase con pregunta.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="B2:C2"/>

</xml_diff>

<commit_message>
docs(acta): filas 71-72 -- diagnostico en una lectura y conexion obsoleta (07/10), /limites y /rankingmod (11/10); base = copia INVERTEX con sus filas 67-70; encabezado al 11/10
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/gerencia/ACTA DE REUNION_PROYECTOS DE DESARROLLO CONFIABILIDAD.xlsx
+++ b/docs/gerencia/ACTA DE REUNION_PROYECTOS DE DESARROLLO CONFIABILIDAD.xlsx
@@ -930,8 +930,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla2" displayName="Tabla2" ref="B19:K66" totalsRowShown="0" headerRowDxfId="14" dataDxfId="12" headerRowBorderDxfId="13" tableBorderDxfId="11" totalsRowBorderDxfId="10">
-  <autoFilter ref="B19:K66" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla2" displayName="Tabla2" ref="B19:K72" totalsRowShown="0" headerRowDxfId="14" dataDxfId="12" headerRowBorderDxfId="13" tableBorderDxfId="11" totalsRowBorderDxfId="10">
+  <autoFilter ref="B19:K72" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Proyecto" dataDxfId="9"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Asunto" dataDxfId="8"/>
@@ -1265,7 +1265,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:K66"/>
+  <dimension ref="B2:K72"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.77734375" customWidth="1"/>
@@ -1303,7 +1303,7 @@
         <v>17</v>
       </c>
       <c r="K4" s="8">
-        <v>46299</v>
+        <v>46306</v>
       </c>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.3">
@@ -2597,7 +2597,7 @@
       </c>
       <c r="K47" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">17/09 - Nuevo botón «Histórico de Metales» en Utilidades (solo desarrollo): recibe la misma plantilla, toma los camiones con Motivo Catastrófico (14) y por cada uno consulta Oil.LaboratoryData para traer TODAS las muestras del motor entre FECHA Inicio y FECHA Cambio, con la FILA COMPLETA (todos los elementos, degradación, horas y textos; se omiten los acumulados derivados y los IDs internos), jerarquizada (identidad, horas, los 7 metales protagonistas, resto de elementos, degradación, lo demás al final). Genera un Excel en FORMATO TABLA con una hoja por camión y una fila ACUMULADO que cuadra con el reporte (3162: Fe 171, Pb 147, Cu 94). ESN desde la BD (respaldo de la plantilla); ODI/POS de la plantilla; celdas sin dato = «null» (distinto de 0.00 medido). Software en v4.8.0.</t>
+          <t xml:space="preserve">17/09 - Nuevo botón «Histórico de Metales» en Utilidades (solo desarrollo): recibe la misma plantilla, toma los camiones con Motivo Catastrófico (14) y por cada uno consulta Oil.LaboratoryData para traer TODAS las muestras del motor entre FECHA Inicio y FECHA Cambio, con la FILA COMPLETA (todos los elementos, degradación, horas y textos; se omiten los acumulados derivados y los IDs internos), jerarquizada (identidad, horas, los 7 metales protagonistas, resto de elementos, degradación, lo demás al final). Genera un Excel en FORMATO TABLA con una hoja por camión y una fila ACUMULADO que cuadra con el reporte (3162: Fe 171, Pb 147, Cu 94). ESN desde la BD (respaldo de la plantilla); ODI/POS de la plantilla; celdas sin dato = «null» (distinto de 0.00 medido). Software en v4.8.0. || 08/10/26 - Extendido a TOROMOCHO y dinamizado: deja de estar atado a Antapaccay. Sin línea base y sin la política de las 1 000 h, contando TODAS las muestras (no solo las de tipo C). Solo se recortan columnas de identidad/horas irremediablemente vacías; los metales y demás parámetros se quedan aunque vengan nulos. El ESN se propaga dentro de la ventana cuando la BD tiene un único serial; en Toromocho no lo hay (0 de 774 muestras) y se dice, en vez de dejar la columna en blanco sin explicación. El código de equipo se resuelve contra la BD en vez de adivinarse: antes CM405 se convertía en CA405, que no existe, y la consulta volvía vacía sin decir por qué.</t>
         </is>
       </c>
     </row>
@@ -3389,7 +3389,7 @@
         </is>
       </c>
     </row>
-    <row r="66" spans="2:11" ht="220" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:11" ht="220" customHeight="41" x14ac:dyDescent="0.3">
       <c r="B66" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">KomfIA</t>
@@ -3425,12 +3425,257 @@
       </c>
       <c r="K66" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Con Carlos (próximo feedback): los hallazgos de carga y límites de la fila 64 (ruedas con límite de otro aceite, componentes sin límites, ISO en 0, etc.) y si el «Acum» del PQ tiene sentido.
+          <t xml:space="preserve">11/10/26 - CERRADOS: diagnóstico completo en una lectura (2,7 s), conexión «obsoleta» (fila 71) y /limites (fila 72). Siguen: feedback de carga con Carlos, «Acum» del PQ, ponderación por parámetro y los pedidos al DBA.
+Con Carlos (próximo feedback): los hallazgos de carga y límites de la fila 64 (ruedas con límite de otro aceite, componentes sin límites, ISO en 0, etc.) y si el «Acum» del PQ tiene sentido.
 En estudio: ponderación por parámetro (ligada al ranking de acumulados); decide si el código de limpieza cuenta para el estado en el panel y el barrido.
 Rendimiento: el diagnóstico completo aún lee la base 7 veces (7-11 s); es el último ajuste del flujo de uso.
 Copilot: la conexión SQL de algunos flujos queda «obsoleta» durante las pruebas y Teams pide reconectar.
 TI / DBA: permiso de solo lectura de métricas (VIEW DATABASE PERFORMANCE STATE) y evaluar el plan de la base.
 A largo plazo: comando /limites, «siguiente paso sugerido» al pie de los módulos de flota y pase con pregunta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" spans="2:11" ht="250" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B67" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INVERTEX 4</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">«Análisis Métricas .tar» — comparador entre camiones y depuración automática del .tar (v4.9.6)</t>
+        </is>
+      </c>
+      <c r="D67" s="8">
+        <v>46298</v>
+      </c>
+      <c r="E67" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Poder apilar varios .tar y comparar un 980E-5 contra un 980E-5SE; y que el .tar se depure solo al cargarlo, sin botón.</t>
+        </is>
+      </c>
+      <c r="F67" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="G67" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="H67" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="I67" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="J67" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="K67" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">03/10/26 - ENTREGADO (v4.9.6, desplegada). El .tar se depura AL CARGARLO, sin botón: los duplicados se descartan por contenido y el resultado se informa en los KPI y en cada submódulo (122 archivos / 13 MB en el .tar de muestra). || COMPARADOR: se apilan varios .tar y se contrastan ficha del camión, inventario por familia y campos; el vocabulario técnico (códigos de falla) se deja en inglés y el resto se traduce. || La vista se reorganizó: sin título redundante, KPI junto al minititulo, y el filtro de fecha avisa «en límite» y «no se puede cruzar» en vez de quedarse quieto sin explicar por qué.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" spans="2:11" ht="250" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B68" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INVERTEX 4</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Geolocalización — el visor de mapas deja de ser Chromium y pasa a dibujar la flota entera (v4.9.7)</t>
+        </is>
+      </c>
+      <c r="D68" s="8">
+        <v>46303</v>
+      </c>
+      <c r="E68" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cerrar de raíz los cierres del módulo de Geolocalización, probando otras herramientas o librerías si hacía falta.</t>
+        </is>
+      </c>
+      <c r="F68" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="G68" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="H68" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="I68" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="J68" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="K68" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">08/10/26 - ENTREGADO (v4.9.7, desplegada). CAUSA: el visor era Chromium embebido y su proceso de render moría en equipos cargados; tres versiones seguidas (4.9.3-4.9.6) pusieron redes para que la caída no se llevara la app. Se cambió a QtLocation, que pinta el propio Qt: no hay proceso aparte que se pueda morir. Medido: 255 MB contra 555 MB, y el .exe baja de 306 a 246 MB al irse Chromium. || CAPACIDAD: los puntos ya no son un objeto por evento, se funden los que comparten píxel, así que los 108 452 eventos reales se dibujan en 12-24 ms por fotograma (antes 175 ms). Con eso cayeron el tope de selección (eran 5 recomendados / 10 duros) y el de 5 000 puntos, también en el mapa del navegador, que pasó a las mismas 5 capas que el visor. || El cartel «Map data not yet available» tenía TRES causas, las tres medidas: Esri se acaba en z17 sobre la mina (Google llega a z21), el zoom pasaba del tope real de cada capa, y Qt cachea las teselas por hueco y no por URL. Pendiente: más pruebas de campo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" spans="2:11" ht="190" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B69" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INVERTEX 4</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Datapacks — preformatos de parámetros guardados con nombre (v4.9.7)</t>
+        </is>
+      </c>
+      <c r="D69" s="8">
+        <v>46303</v>
+      </c>
+      <c r="E69" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Guardar una selección de señales con nombre («Voltajes») y volver a aplicarla en sesiones siguientes sin marcarlas una a una.</t>
+        </is>
+      </c>
+      <c r="F69" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="G69" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="H69" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="I69" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="J69" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="K69" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">08/10/26 - ENTREGADO. Se guardan en %LOCALAPPDATA%\INVERTEX\preformatos_datapack.json, copiable a otro equipo. Si el datapack no trae alguna señal —modelos distintos graban señales distintas— marca las que hay y lo dice, en vez de marcar de menos en silencio. || Al estrenarlo el botón no hacía NADA: faltaba importar el diálogo del nombre y Qt se traga las excepciones dentro de un slot, así que no había ni error ni aviso. Corregido y cubierto con prueba; se barrió el resto del código buscando el mismo tipo de fallo y no había ninguno más.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" spans="2:11" ht="250" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B70" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INVERTEX 4</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tema de la aplicación — tres paletas y el azul de marca deja de dominar (v4.9.8)</t>
+        </is>
+      </c>
+      <c r="D70" s="8">
+        <v>46303</v>
+      </c>
+      <c r="E70" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Un botón de tema en el vestíbulo con tres paletas (la oscura actual, una Komatsu Mitsui clara y una minimalista), aplicado a TODA la app, y que el azul de marca deje de teñirlo todo.</t>
+        </is>
+      </c>
+      <c r="F70" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="G70" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="H70" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="I70" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="J70" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="K70" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">08/10/26 - ENTREGADO (v4.9.8, desplegada). Komatsu Mitsui está calcado de los reportes del área: banda azul de marca arriba y cuerpo BLANCO, con el azul como acento y no como fondo. Minimalista es claro cálido y lleva tipografía propia, que es lo que de verdad lo separa de «otro tema claro». Profesional queda como el de por defecto y el refugio. || El azul #12239E era a la vez el fondo, el color primario, el marco y la navegación: por eso teñía la app entera. Ya no lo es en ninguno de los tres temas. Se repasaron los 11 módulos en las tres paletas, y cada subvista de Geolocalización se pinta en su propio color (marrón, verde, azul marino). || De paso salieron dos cosas: el perfil de velocidad bajó de 18,5 s a 1,2 s —entrar al módulo recorría los 319 datapacks del .tar para acabar fallando, porque ese camión no graba gps_speed_mph— y los iconos de las gráficas, que salían blancos sobre fondo claro. || PENDIENTE: las fotos del vestíbulo y el logo del núcleo siguen siendo assets azules; para un Komatsu pleno harían falta versiones claras.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" spans="2:11" ht="170" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B71" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KomfIA</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Diagnóstico completo en una sola lectura y la conexión que Teams pedía reconectar</t>
+        </is>
+      </c>
+      <c r="D71" s="8">
+        <v>46302</v>
+      </c>
+      <c r="E71" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cerrar los dos pendientes técnicos que quedaron del 04/10: el diagnóstico completo seguía lento y, una o dos veces al mes, Teams pedía reconectar la conexión de un comando.</t>
+        </is>
+      </c>
+      <c r="F71" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="G71" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="H71" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="I71" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="J71" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="K71" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">07/10/26 - HECHO. Diagnóstico completo de un equipo: de 19,5 s a 2,7 s (y el diagnóstico de observados de 25,5 s a 2,9 s). La vista leía la base 9 veces, una por cada parte de la tabla; ahora la lee una sola vez y entrega exactamente lo mismo. Al comparar salió que en HT079 (Antamina) aparecen dos columnas «MT RH»: es el componente mal escrito «MOTORO DE TRACCION RH», que sigue entrando a la base (pendiente de carga con Carlos).
+Conexión «Obsoleta»: la base de datos estaba bien configurada; el flujo del ranking pedía la conexión de cada usuario en vez de usar la del creador, y ese permiso caducaba. Corregido: en producción nadie verá esa tarjeta. Revisado el resto de flujos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" spans="2:11" ht="230" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B72" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KomfIA</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Comando /limites y /limitesc — la tabla de límites del área, completa y filtrable</t>
+        </is>
+      </c>
+      <c r="D72" s="8">
+        <v>46306</v>
+      </c>
+      <c r="E72" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Consultar los límites (LP/LC) tal como están cargados por el área, con todos los parámetros que realmente los tienen, y poder filtrar por mina, flota, componente y uno o varios parámetros. Era el último pendiente aparcado de la presentación del 02/10.</t>
+        </is>
+      </c>
+      <c r="F72" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="G72" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="H72" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="I72" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="J72" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="K72" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">11/10/26 - ENTREGADO y probado en Teams. Una tabla por modelo: parámetros en filas, componentes en columnas (MT LH, MT RH, sistema hidráulico, motor, ruedas, y también mando final, transmisión, PTO, caja de giro y damper). /limites muestra solo los parámetros con límite; /limitesc, el formato completo con «—» donde falta.
+Ejemplos: «/limites traccion Fe,Cu,Pb», «/limites antamina motor TBN», «/limitesc antapaccay 980». Por defecto: Antapaccay, todo. Si un parámetro no tiene límite lo dice y sugiere /limitesc. También responde en lenguaje natural («qué límites tiene el hidráulico del 980E»).
+Aparecen límites que ningún módulo mostraba: cadmio, vanadio, plata, antimonio, litio y glicol (KomfIA no los evalúa todavía). La tabla incluye además a Quellaveco, que está cargada aunque no es parte del alcance.
+De paso: el ranking de acumulados del motor diésel pasa a llamarse /rankingmod (/rankingacum sigue funcionando) y deja el nombre libre para los acumulados por componente.</t>
         </is>
       </c>
     </row>

</xml_diff>